<commit_message>
docs(qc): ship TG portal design-QC report and update shared tracker
Updated QC report PDF, HTML, audit-master.json, and report-sections.json
for the National Portal for Transgender Persons (31 screens, 33 findings).
Refreshed build_final_report.py with per-screen finding arrays and multi-
group global findings. Updated the shared MoSJE-Portal-QC-Tracker.xlsx
with the TG portal findings sheet and rollup row.
</commit_message>
<xml_diff>
--- a/docs/qc/MoSJE-Portal-QC-Tracker.xlsx
+++ b/docs/qc/MoSJE-Portal-QC-Tracker.xlsx
@@ -12,13 +12,17 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="eUtthan Admin" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NHAPOA" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage – NHAPOA" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage – eUtthan" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TG" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage – TG" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage – eUtthan" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'eUtthan Admin'!$A$1:$L$400</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'NHAPOA'!$A$1:$M$152</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Coverage – NHAPOA'!$A$1:$H$81</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Coverage – eUtthan'!$A$1:$H$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'TG'!$A$1:$M$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Coverage – TG'!$A$1:$H$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Coverage – eUtthan'!$A$1:$H$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -841,7 +845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -989,7 +993,46 @@
         <v/>
       </c>
     </row>
-    <row r="7"/>
+    <row r="7">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>TG</t>
+        </is>
+      </c>
+      <c r="B7" s="19">
+        <f>COUNTA('TG'!$A$2:$A$400)</f>
+        <v/>
+      </c>
+      <c r="C7" s="19">
+        <f>COUNTIF('TG'!$D:$D,"Blocker")</f>
+        <v/>
+      </c>
+      <c r="D7" s="19">
+        <f>COUNTIF('TG'!$D:$D,"Major")</f>
+        <v/>
+      </c>
+      <c r="E7" s="19">
+        <f>COUNTIF('TG'!$D:$D,"Minor")</f>
+        <v/>
+      </c>
+      <c r="F7" s="19">
+        <f>COUNTIF('TG'!$D:$D,"Nit")</f>
+        <v/>
+      </c>
+      <c r="G7" s="19">
+        <f>COUNTIF('TG'!$I:$I,"Open")</f>
+        <v/>
+      </c>
+      <c r="H7" s="19">
+        <f>COUNTIF('TG'!$I:$I,"Fixed")</f>
+        <v/>
+      </c>
+      <c r="I7" s="19">
+        <f>COUNTIF('TG'!$I:$I,"Verified")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -20561,6 +20604,3320 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:M34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="20" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+      <c r="C1" s="20" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D1" s="20" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="E1" s="20" t="inlineStr">
+        <is>
+          <t>Issue (Design → Built)</t>
+        </is>
+      </c>
+      <c r="F1" s="20" t="inlineStr">
+        <is>
+          <t>Recommended Fix (Dev)</t>
+        </is>
+      </c>
+      <c r="G1" s="20" t="inlineStr">
+        <is>
+          <t>Figma URL</t>
+        </is>
+      </c>
+      <c r="H1" s="20" t="inlineStr">
+        <is>
+          <t>Live URL</t>
+        </is>
+      </c>
+      <c r="I1" s="20" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="J1" s="20" t="inlineStr">
+        <is>
+          <t>Assignee</t>
+        </is>
+      </c>
+      <c r="K1" s="20" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="L1" s="20" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="M1" s="20" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="21" t="inlineStr">
+        <is>
+          <t>TG-GLOBAL-001</t>
+        </is>
+      </c>
+      <c r="B2" s="21" t="inlineStr">
+        <is>
+          <t>Global · Government masthead · dashboards · tables</t>
+        </is>
+      </c>
+      <c r="C2" s="21" t="inlineStr">
+        <is>
+          <t>Content &amp; Iconography</t>
+        </is>
+      </c>
+      <c r="D2" s="21" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="E2" s="21" t="inlineStr">
+        <is>
+          <t>Figma: The masthead right zone carries the SAMAVESH co-branding lockup — the Digital India logo + the SAMAVESH logo — before the user/avatar block.  →  Live: Both logos are omitted portal-wide; only the user name/role/avatar remain on the right. (Present on the login hero, missing on every authenticated inner page.)</t>
+        </is>
+      </c>
+      <c r="F2" s="21" t="inlineStr">
+        <is>
+          <t>Restore the Digital India + SAMAVESH co-branding lockup in the masthead right zone per the design, on every screen.</t>
+        </is>
+      </c>
+      <c r="G2" s="22" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-38830</t>
+        </is>
+      </c>
+      <c r="H2" s="22" t="inlineStr">
+        <is>
+          <t>https://tg-admin-dev.mosje.in/dashboard</t>
+        </is>
+      </c>
+      <c r="I2" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J2" s="21" t="inlineStr"/>
+      <c r="K2" s="21" t="inlineStr"/>
+      <c r="L2" s="21" t="inlineStr">
+        <is>
+          <t>env: dev  ·  Scope: Global — these elements repeat across the portal; fix once. The board shows a representative frame (Central Admin — Dashboard) — open it via 'Figma frame ↗'; each marker's number matches its TG-GLOBAL id.</t>
+        </is>
+      </c>
+      <c r="M2" s="21" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="23" t="inlineStr">
+        <is>
+          <t>TG-GLOBAL-002</t>
+        </is>
+      </c>
+      <c r="B3" s="23" t="inlineStr">
+        <is>
+          <t>Global · Government masthead · dashboards · tables</t>
+        </is>
+      </c>
+      <c r="C3" s="23" t="inlineStr">
+        <is>
+          <t>Content &amp; Iconography</t>
+        </is>
+      </c>
+      <c r="D3" s="23" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E3" s="23" t="inlineStr">
+        <is>
+          <t>Figma: 'Government of India / Ministry of Social Justice &amp; Empowerment / Department of Social Justice &amp; Empowerment' (Department line in bold navy).  →  Live: Only 'Government of India / Ministry of Social Justice &amp; Empowerment' — the Department line is dropped and the bold weight moves up a line.</t>
+        </is>
+      </c>
+      <c r="F3" s="23" t="inlineStr">
+        <is>
+          <t>Render the full 3-line identity lockup with the Department line bold, per the design masthead.</t>
+        </is>
+      </c>
+      <c r="G3" s="24" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-38830</t>
+        </is>
+      </c>
+      <c r="H3" s="24" t="inlineStr">
+        <is>
+          <t>https://tg-admin-dev.mosje.in/dashboard</t>
+        </is>
+      </c>
+      <c r="I3" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J3" s="23" t="inlineStr"/>
+      <c r="K3" s="23" t="inlineStr"/>
+      <c r="L3" s="23" t="inlineStr">
+        <is>
+          <t>env: dev  ·  Scope: Global — these elements repeat across the portal; fix once. The board shows a representative frame (Central Admin — Dashboard) — open it via 'Figma frame ↗'; each marker's number matches its TG-GLOBAL id.</t>
+        </is>
+      </c>
+      <c r="M3" s="23" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="21" t="inlineStr">
+        <is>
+          <t>TG-GLOBAL-003</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>Global · Government masthead · dashboards · tables</t>
+        </is>
+      </c>
+      <c r="C4" s="21" t="inlineStr">
+        <is>
+          <t>Components &amp; States</t>
+        </is>
+      </c>
+      <c r="D4" s="21" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="E4" s="21" t="inlineStr">
+        <is>
+          <t>Figma: Each dashboard KPI card shows a leading metric icon and a delta/trend line ('▲ +14.5% vs last month' or a contextual subtitle).  →  Live: KPI cards render only a label + number — the icon and trend/subtext are dropped, losing the at-a-glance comparison hierarchy.</t>
+        </is>
+      </c>
+      <c r="F4" s="21" t="inlineStr">
+        <is>
+          <t>Restore the KPI card icon and trend/delta subtitle per the design KPI component. Applies to all role dashboards.</t>
+        </is>
+      </c>
+      <c r="G4" s="22" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-38830</t>
+        </is>
+      </c>
+      <c r="H4" s="22" t="inlineStr">
+        <is>
+          <t>https://tg-admin-dev.mosje.in/dashboard</t>
+        </is>
+      </c>
+      <c r="I4" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J4" s="21" t="inlineStr"/>
+      <c r="K4" s="21" t="inlineStr"/>
+      <c r="L4" s="21" t="inlineStr">
+        <is>
+          <t>env: dev  ·  Scope: Global — these elements repeat across the portal; fix once. The board shows a representative frame (Central Admin — Dashboard) — open it via 'Figma frame ↗'; each marker's number matches its TG-GLOBAL id.</t>
+        </is>
+      </c>
+      <c r="M4" s="21" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t>TG-GLOBAL-004</t>
+        </is>
+      </c>
+      <c r="B5" s="23" t="inlineStr">
+        <is>
+          <t>Global · Government masthead · dashboards · tables</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="inlineStr">
+        <is>
+          <t>Components &amp; States</t>
+        </is>
+      </c>
+      <c r="D5" s="23" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E5" s="23" t="inlineStr">
+        <is>
+          <t>Figma: Active page = outlined (white fill, navy border, navy numeral).  →  Live: Active page = a navy-filled chip with a white numeral.</t>
+        </is>
+      </c>
+      <c r="F5" s="23" t="inlineStr">
+        <is>
+          <t>Match the pagination active-page control to the design's outlined style. Applies to every paginated table.</t>
+        </is>
+      </c>
+      <c r="G5" s="24" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-38830</t>
+        </is>
+      </c>
+      <c r="H5" s="24" t="inlineStr">
+        <is>
+          <t>https://tg-admin-dev.mosje.in/dashboard</t>
+        </is>
+      </c>
+      <c r="I5" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J5" s="23" t="inlineStr"/>
+      <c r="K5" s="23" t="inlineStr"/>
+      <c r="L5" s="23" t="inlineStr">
+        <is>
+          <t>env: dev  ·  Scope: Global — these elements repeat across the portal; fix once. The board shows a representative frame (Central Admin — Dashboard) — open it via 'Figma frame ↗'; each marker's number matches its TG-GLOBAL id.</t>
+        </is>
+      </c>
+      <c r="M5" s="23" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>TG-GLOBAL-005</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>Global · Government masthead · dashboards · tables</t>
+        </is>
+      </c>
+      <c r="C6" s="21" t="inlineStr">
+        <is>
+          <t>Color &amp; Token</t>
+        </is>
+      </c>
+      <c r="D6" s="21" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E6" s="21" t="inlineStr">
+        <is>
+          <t>Figma: Table headers use a light neutral-gray fill (≈#f9fafb, Stroke/50).  →  Live: Dashboard queue tables use a near-neutral header, but the User/Role/Tenant management tables use a light blue header tint (≈#dbeafe).</t>
+        </is>
+      </c>
+      <c r="F6" s="21" t="inlineStr">
+        <is>
+          <t>Standardise all data-table headers to the neutral-gray header token; drop the blue tint on the management tables.</t>
+        </is>
+      </c>
+      <c r="G6" s="22" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-38830</t>
+        </is>
+      </c>
+      <c r="H6" s="22" t="inlineStr">
+        <is>
+          <t>https://tg-admin-dev.mosje.in/dashboard</t>
+        </is>
+      </c>
+      <c r="I6" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J6" s="21" t="inlineStr"/>
+      <c r="K6" s="21" t="inlineStr"/>
+      <c r="L6" s="21" t="inlineStr">
+        <is>
+          <t>env: dev  ·  Scope: Global — these elements repeat across the portal; fix once. The board shows a representative frame (Central Admin — Dashboard) — open it via 'Figma frame ↗'; each marker's number matches its TG-GLOBAL id.</t>
+        </is>
+      </c>
+      <c r="M6" s="21" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t>TG-GLOBAL-006</t>
+        </is>
+      </c>
+      <c r="B7" s="23" t="inlineStr">
+        <is>
+          <t>Global · Application review — validation &amp; documents</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="inlineStr">
+        <is>
+          <t>Components &amp; States</t>
+        </is>
+      </c>
+      <c r="D7" s="23" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="E7" s="23" t="inlineStr">
+        <is>
+          <t>Figma: System Validation lists three checks — Data Validation, Duplicate Check (with the match + similarity score, e.g. 'Potential match: TG2024-LU-04521 (85% similarity)') and Document Verification.  →  Live: The build shows only Data Validation and Document Verification — the Duplicate Check row is absent, so the duplicate-detection signal never reaches the reviewer. Repeats on every role's application review screen.</t>
+        </is>
+      </c>
+      <c r="F7" s="23" t="inlineStr">
+        <is>
+          <t>Restore the Duplicate Check row in System Validation with its match reference + similarity status. Applies to every role's application review screen.</t>
+        </is>
+      </c>
+      <c r="G7" s="24" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-39123</t>
+        </is>
+      </c>
+      <c r="H7" s="24" t="inlineStr">
+        <is>
+          <t>https://tg-admin-dev.mosje.in/applications</t>
+        </is>
+      </c>
+      <c r="I7" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J7" s="23" t="inlineStr"/>
+      <c r="K7" s="23" t="inlineStr"/>
+      <c r="L7" s="23" t="inlineStr">
+        <is>
+          <t>env: dev  ·  Scope: Global — these elements repeat across the portal; fix once. The board shows a representative frame (Examining Officer — Application Documents) — open it via 'Figma frame ↗'; each marker's number matches its TG-GLOBAL id.</t>
+        </is>
+      </c>
+      <c r="M7" s="23" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>TG-GLOBAL-007</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>Global · Application review — validation &amp; documents</t>
+        </is>
+      </c>
+      <c r="C8" s="21" t="inlineStr">
+        <is>
+          <t>Content &amp; Iconography</t>
+        </is>
+      </c>
+      <c r="D8" s="21" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="E8" s="21" t="inlineStr">
+        <is>
+          <t>Figma: Each document is listed by its semantic name — 'Signed Affidavit', 'Aadhaar Card', 'Passport Photo' — with a matching document-type icon.  →  Live: The build lists raw upload filenames ('form1 (2).pdf', 'Screenshot 2026-06-24 221031.pdf', 'tgportal-image.jpg') against a generic file glyph, so a reviewer cannot tell which document is which without opening each one. Repeats on every role's Documents tab.</t>
+        </is>
+      </c>
+      <c r="F8" s="21" t="inlineStr">
+        <is>
+          <t>Label each document by its semantic type with the matching type icon and keep the filename as secondary text. Applies to every role's Documents tab.</t>
+        </is>
+      </c>
+      <c r="G8" s="22" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-39123</t>
+        </is>
+      </c>
+      <c r="H8" s="22" t="inlineStr">
+        <is>
+          <t>https://tg-admin-dev.mosje.in/applications</t>
+        </is>
+      </c>
+      <c r="I8" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J8" s="21" t="inlineStr"/>
+      <c r="K8" s="21" t="inlineStr"/>
+      <c r="L8" s="21" t="inlineStr">
+        <is>
+          <t>env: dev  ·  Scope: Global — these elements repeat across the portal; fix once. The board shows a representative frame (Examining Officer — Application Documents) — open it via 'Figma frame ↗'; each marker's number matches its TG-GLOBAL id.</t>
+        </is>
+      </c>
+      <c r="M8" s="21" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="23" t="inlineStr">
+        <is>
+          <t>TG-GLOBAL-008</t>
+        </is>
+      </c>
+      <c r="B9" s="23" t="inlineStr">
+        <is>
+          <t>Global · Application review — validation &amp; documents</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="inlineStr">
+        <is>
+          <t>Components &amp; States</t>
+        </is>
+      </c>
+      <c r="D9" s="23" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E9" s="23" t="inlineStr">
+        <is>
+          <t>Figma: When the system detects a similar record the screen surfaces an amber 'Exception Flagged: Duplicate' banner above the application, explaining the match.  →  Live: The build never renders the exception banner, so flagged applications look identical to clean ones.</t>
+        </is>
+      </c>
+      <c r="F9" s="23" t="inlineStr">
+        <is>
+          <t>Render the exception banner when the duplicate/exception check trips, per the design.</t>
+        </is>
+      </c>
+      <c r="G9" s="24" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-39123</t>
+        </is>
+      </c>
+      <c r="H9" s="24" t="inlineStr">
+        <is>
+          <t>https://tg-admin-dev.mosje.in/applications</t>
+        </is>
+      </c>
+      <c r="I9" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J9" s="23" t="inlineStr"/>
+      <c r="K9" s="23" t="inlineStr"/>
+      <c r="L9" s="23" t="inlineStr">
+        <is>
+          <t>env: dev  ·  Scope: Global — these elements repeat across the portal; fix once. The board shows a representative frame (Examining Officer — Application Documents) — open it via 'Figma frame ↗'; each marker's number matches its TG-GLOBAL id.</t>
+        </is>
+      </c>
+      <c r="M9" s="23" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>TG-CIT-SIGNIN-001</t>
+        </is>
+      </c>
+      <c r="B10" s="21" t="inlineStr">
+        <is>
+          <t>Citizen — Sign In</t>
+        </is>
+      </c>
+      <c r="C10" s="21" t="inlineStr">
+        <is>
+          <t>Components &amp; States</t>
+        </is>
+      </c>
+      <c r="D10" s="21" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="E10" s="21" t="inlineStr">
+        <is>
+          <t>Figma: The login card leads with a three-way role switcher — Citizen · Admin · Garima Greh — with Citizen active.  →  Live: The citizen build renders no role tabs; the card opens straight into the 'Log In to your account' heading.</t>
+        </is>
+      </c>
+      <c r="F10" s="21" t="inlineStr">
+        <is>
+          <t>Restore the Citizen / Admin / Garima Greh role-tab switcher at the top of the login card, per the design frame.</t>
+        </is>
+      </c>
+      <c r="G10" s="22" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=9379-115794</t>
+        </is>
+      </c>
+      <c r="H10" s="22" t="inlineStr">
+        <is>
+          <t>https://tg-user-dev.mosje.in/auth/sign-in</t>
+        </is>
+      </c>
+      <c r="I10" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J10" s="21" t="inlineStr"/>
+      <c r="K10" s="21" t="inlineStr"/>
+      <c r="L10" s="21" t="inlineStr">
+        <is>
+          <t>env: dev</t>
+        </is>
+      </c>
+      <c r="M10" s="21" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="23" t="inlineStr">
+        <is>
+          <t>TG-CIT-SIGNIN-002</t>
+        </is>
+      </c>
+      <c r="B11" s="23" t="inlineStr">
+        <is>
+          <t>Citizen — Sign In</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>Components &amp; States</t>
+        </is>
+      </c>
+      <c r="D11" s="23" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="E11" s="23" t="inlineStr">
+        <is>
+          <t>Figma: The design offers a single Email field under 'or sign in with credentials', then a Send OTP button.  →  Live: The build inserts a second 'Mobile Number' field (with its own 'or' divider) below the Email Id field — absent from the design.</t>
+        </is>
+      </c>
+      <c r="F11" s="23" t="inlineStr">
+        <is>
+          <t>Align to the design's single-field pattern, or update the design frame if the Mobile Number entry is a deliberate addition.</t>
+        </is>
+      </c>
+      <c r="G11" s="24" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=9379-115794</t>
+        </is>
+      </c>
+      <c r="H11" s="24" t="inlineStr">
+        <is>
+          <t>https://tg-user-dev.mosje.in/auth/sign-in</t>
+        </is>
+      </c>
+      <c r="I11" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J11" s="23" t="inlineStr"/>
+      <c r="K11" s="23" t="inlineStr"/>
+      <c r="L11" s="23" t="inlineStr">
+        <is>
+          <t>env: dev</t>
+        </is>
+      </c>
+      <c r="M11" s="23" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>TG-CIT-SIGNIN-003</t>
+        </is>
+      </c>
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>Citizen — Sign In</t>
+        </is>
+      </c>
+      <c r="C12" s="21" t="inlineStr">
+        <is>
+          <t>Typography</t>
+        </is>
+      </c>
+      <c r="D12" s="21" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E12" s="21" t="inlineStr">
+        <is>
+          <t>Figma: The heading reads 'Log in to your account' (sentence case).  →  Live: The build renders 'Log In to your account' — 'In' is capitalised.</t>
+        </is>
+      </c>
+      <c r="F12" s="21" t="inlineStr">
+        <is>
+          <t>Match the design's sentence-case heading: 'Log in to your account'.</t>
+        </is>
+      </c>
+      <c r="G12" s="22" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=9379-115794</t>
+        </is>
+      </c>
+      <c r="H12" s="22" t="inlineStr">
+        <is>
+          <t>https://tg-user-dev.mosje.in/auth/sign-in</t>
+        </is>
+      </c>
+      <c r="I12" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J12" s="21" t="inlineStr"/>
+      <c r="K12" s="21" t="inlineStr"/>
+      <c r="L12" s="21" t="inlineStr">
+        <is>
+          <t>env: dev</t>
+        </is>
+      </c>
+      <c r="M12" s="21" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="inlineStr">
+        <is>
+          <t>TG-ADM-SIGNIN-001</t>
+        </is>
+      </c>
+      <c r="B13" s="23" t="inlineStr">
+        <is>
+          <t>Admin — Log In</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>Components &amp; States</t>
+        </is>
+      </c>
+      <c r="D13" s="23" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="E13" s="23" t="inlineStr">
+        <is>
+          <t>Figma: The design offers a single Email field, then a Send OTP button.  →  Live: The build adds a second 'Mobile Number' field (with an 'or' divider) below Email — absent from the design.</t>
+        </is>
+      </c>
+      <c r="F13" s="23" t="inlineStr">
+        <is>
+          <t>Align to the design's single Email-field pattern, or update the design frame if Mobile Number entry is a deliberate addition.</t>
+        </is>
+      </c>
+      <c r="G13" s="24" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=9387-138143</t>
+        </is>
+      </c>
+      <c r="H13" s="24" t="inlineStr">
+        <is>
+          <t>https://tg-admin-dev.mosje.in/login</t>
+        </is>
+      </c>
+      <c r="I13" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J13" s="23" t="inlineStr"/>
+      <c r="K13" s="23" t="inlineStr"/>
+      <c r="L13" s="23" t="inlineStr">
+        <is>
+          <t>env: dev</t>
+        </is>
+      </c>
+      <c r="M13" s="23" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="21" t="inlineStr">
+        <is>
+          <t>TG-ADM-SIGNIN-002</t>
+        </is>
+      </c>
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <t>Admin — Log In</t>
+        </is>
+      </c>
+      <c r="C14" s="21" t="inlineStr">
+        <is>
+          <t>Typography</t>
+        </is>
+      </c>
+      <c r="D14" s="21" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E14" s="21" t="inlineStr">
+        <is>
+          <t>Figma: The heading reads 'Log in to your account' (sentence case).  →  Live: The build renders 'Log In to your account' — 'In' is capitalised.</t>
+        </is>
+      </c>
+      <c r="F14" s="21" t="inlineStr">
+        <is>
+          <t>Match the design's sentence-case heading: 'Log in to your account'.</t>
+        </is>
+      </c>
+      <c r="G14" s="22" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=9387-138143</t>
+        </is>
+      </c>
+      <c r="H14" s="22" t="inlineStr">
+        <is>
+          <t>https://tg-admin-dev.mosje.in/login</t>
+        </is>
+      </c>
+      <c r="I14" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J14" s="21" t="inlineStr"/>
+      <c r="K14" s="21" t="inlineStr"/>
+      <c r="L14" s="21" t="inlineStr">
+        <is>
+          <t>env: dev</t>
+        </is>
+      </c>
+      <c r="M14" s="21" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>TG-CIT-APPLY-IDENTITY-001</t>
+        </is>
+      </c>
+      <c r="B15" s="23" t="inlineStr">
+        <is>
+          <t>Citizen — Apply · Step 1 · Basic Identity Details</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
+          <t>Layout &amp; Spacing</t>
+        </is>
+      </c>
+      <c r="D15" s="23" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E15" s="23" t="inlineStr">
+        <is>
+          <t>Figma: Self-Perceived Identity and Permanent Address lay out on a 3-column field grid.  →  Live: The build uses a 2-column grid, making the form noticeably taller and pushing the primary action below the fold.</t>
+        </is>
+      </c>
+      <c r="F15" s="23" t="inlineStr">
+        <is>
+          <t>Match the design's 3-column field grid on the identity step.</t>
+        </is>
+      </c>
+      <c r="G15" s="24" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=3531-35553</t>
+        </is>
+      </c>
+      <c r="H15" s="24" t="inlineStr">
+        <is>
+          <t>https://tg-user-dev.mosje.in/apply</t>
+        </is>
+      </c>
+      <c r="I15" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J15" s="23" t="inlineStr"/>
+      <c r="K15" s="23" t="inlineStr"/>
+      <c r="L15" s="23" t="inlineStr">
+        <is>
+          <t>env: dev</t>
+        </is>
+      </c>
+      <c r="M15" s="23" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>TG-CIT-APPLY-IDENTITY-002</t>
+        </is>
+      </c>
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>Citizen — Apply · Step 1 · Basic Identity Details</t>
+        </is>
+      </c>
+      <c r="C16" s="21" t="inlineStr">
+        <is>
+          <t>Components &amp; States</t>
+        </is>
+      </c>
+      <c r="D16" s="21" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E16" s="21" t="inlineStr">
+        <is>
+          <t>Figma: A single checkbox reads 'My Current / Correspondence address is the same as my Permanent address.'  →  Live: The build asks 'Is your correspondence address the same as your permanent address?' with Yes/No toggle buttons.</t>
+        </is>
+      </c>
+      <c r="F16" s="21" t="inlineStr">
+        <is>
+          <t>Use the design's single checkbox for the correspondence-address control.</t>
+        </is>
+      </c>
+      <c r="G16" s="22" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=3531-35553</t>
+        </is>
+      </c>
+      <c r="H16" s="22" t="inlineStr">
+        <is>
+          <t>https://tg-user-dev.mosje.in/apply</t>
+        </is>
+      </c>
+      <c r="I16" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J16" s="21" t="inlineStr"/>
+      <c r="K16" s="21" t="inlineStr"/>
+      <c r="L16" s="21" t="inlineStr">
+        <is>
+          <t>env: dev</t>
+        </is>
+      </c>
+      <c r="M16" s="21" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="23" t="inlineStr">
+        <is>
+          <t>TG-CIT-APPLY-IDENTITY-003</t>
+        </is>
+      </c>
+      <c r="B17" s="23" t="inlineStr">
+        <is>
+          <t>Citizen — Apply · Step 1 · Basic Identity Details</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="inlineStr">
+        <is>
+          <t>Components &amp; States</t>
+        </is>
+      </c>
+      <c r="D17" s="23" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E17" s="23" t="inlineStr">
+        <is>
+          <t>Figma: The bottom-left control on the step is 'Cancel'.  →  Live: The build renders 'Back' instead.</t>
+        </is>
+      </c>
+      <c r="F17" s="23" t="inlineStr">
+        <is>
+          <t>Relabel the bottom-left control to 'Cancel' per the design.</t>
+        </is>
+      </c>
+      <c r="G17" s="24" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=3531-35553</t>
+        </is>
+      </c>
+      <c r="H17" s="24" t="inlineStr">
+        <is>
+          <t>https://tg-user-dev.mosje.in/apply</t>
+        </is>
+      </c>
+      <c r="I17" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J17" s="23" t="inlineStr"/>
+      <c r="K17" s="23" t="inlineStr"/>
+      <c r="L17" s="23" t="inlineStr">
+        <is>
+          <t>env: dev</t>
+        </is>
+      </c>
+      <c r="M17" s="23" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>TG-CIT-APPLY-IDENTITY-004</t>
+        </is>
+      </c>
+      <c r="B18" s="21" t="inlineStr">
+        <is>
+          <t>Citizen — Apply · Step 1 · Basic Identity Details</t>
+        </is>
+      </c>
+      <c r="C18" s="21" t="inlineStr">
+        <is>
+          <t>Components &amp; States</t>
+        </is>
+      </c>
+      <c r="D18" s="21" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E18" s="21" t="inlineStr">
+        <is>
+          <t>Figma: The active step is a solid navy disc with a white numeral.  →  Live: The build renders the active step as an outlined ring, so it reads like an inactive step.</t>
+        </is>
+      </c>
+      <c r="F18" s="21" t="inlineStr">
+        <is>
+          <t>Give the active step the design's solid navy fill + white numeral.</t>
+        </is>
+      </c>
+      <c r="G18" s="22" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=3531-35553</t>
+        </is>
+      </c>
+      <c r="H18" s="22" t="inlineStr">
+        <is>
+          <t>https://tg-user-dev.mosje.in/apply</t>
+        </is>
+      </c>
+      <c r="I18" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J18" s="21" t="inlineStr"/>
+      <c r="K18" s="21" t="inlineStr"/>
+      <c r="L18" s="21" t="inlineStr">
+        <is>
+          <t>env: dev</t>
+        </is>
+      </c>
+      <c r="M18" s="21" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="23" t="inlineStr">
+        <is>
+          <t>TG-CIT-DASH-001</t>
+        </is>
+      </c>
+      <c r="B19" s="23" t="inlineStr">
+        <is>
+          <t>Citizen — Dashboard · Certificate Active</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="inlineStr">
+        <is>
+          <t>Layout &amp; Spacing</t>
+        </is>
+      </c>
+      <c r="D19" s="23" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E19" s="23" t="inlineStr">
+        <is>
+          <t>Figma: All four benefit cards — Scholarships, Skill Training, Garima Greh, Medical Support — sit in a single 4-up row.  →  Live: The build's cards are wider, so only three fit and Medical Support wraps onto a second row.</t>
+        </is>
+      </c>
+      <c r="F19" s="23" t="inlineStr">
+        <is>
+          <t>Match the design's 4-up Welfare Benefits grid so the row doesn't wrap.</t>
+        </is>
+      </c>
+      <c r="G19" s="24" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=3531-36919</t>
+        </is>
+      </c>
+      <c r="H19" s="24" t="inlineStr">
+        <is>
+          <t>https://tg-user-dev.mosje.in/dashboard</t>
+        </is>
+      </c>
+      <c r="I19" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J19" s="23" t="inlineStr"/>
+      <c r="K19" s="23" t="inlineStr"/>
+      <c r="L19" s="23" t="inlineStr">
+        <is>
+          <t>env: dev</t>
+        </is>
+      </c>
+      <c r="M19" s="23" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t>TG-CIT-DASH-002</t>
+        </is>
+      </c>
+      <c r="B20" s="21" t="inlineStr">
+        <is>
+          <t>Citizen — Dashboard · Certificate Active</t>
+        </is>
+      </c>
+      <c r="C20" s="21" t="inlineStr">
+        <is>
+          <t>Components &amp; States</t>
+        </is>
+      </c>
+      <c r="D20" s="21" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E20" s="21" t="inlineStr">
+        <is>
+          <t>Figma: The sidebar lists Dashboard / Certificate/ID / Scholarships / Grievances, each with a leading icon.  →  Live: The build's sidebar has no per-item icons and drops the Scholarships entry (it shows a 'Transgender' scheme dropdown above the list instead).</t>
+        </is>
+      </c>
+      <c r="F20" s="21" t="inlineStr">
+        <is>
+          <t>Restore the per-item sidebar icons and the Scholarships nav entry per the design.</t>
+        </is>
+      </c>
+      <c r="G20" s="22" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=3531-36919</t>
+        </is>
+      </c>
+      <c r="H20" s="22" t="inlineStr">
+        <is>
+          <t>https://tg-user-dev.mosje.in/dashboard</t>
+        </is>
+      </c>
+      <c r="I20" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J20" s="21" t="inlineStr"/>
+      <c r="K20" s="21" t="inlineStr"/>
+      <c r="L20" s="21" t="inlineStr">
+        <is>
+          <t>env: dev</t>
+        </is>
+      </c>
+      <c r="M20" s="21" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="23" t="inlineStr">
+        <is>
+          <t>TG-CIT-CERT-DETAIL-001</t>
+        </is>
+      </c>
+      <c r="B21" s="23" t="inlineStr">
+        <is>
+          <t>Citizen — Certificate &amp; Identity Card</t>
+        </is>
+      </c>
+      <c r="C21" s="23" t="inlineStr">
+        <is>
+          <t>Components &amp; States</t>
+        </is>
+      </c>
+      <c r="D21" s="23" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="E21" s="23" t="inlineStr">
+        <is>
+          <t>Figma: The certificate page carries an OTHER SERVICES section with four lifecycle actions — New Transgender Certificate &amp; ID, Revised Certificate (Post-Medical Intervention), Correction or Update Existing Details, and Withdraw a Pending Application.  →  Live: The build renders the dashboard's Welfare Benefits cards here instead, so none of the certificate lifecycle actions are reachable from this page.</t>
+        </is>
+      </c>
+      <c r="F21" s="23" t="inlineStr">
+        <is>
+          <t>Restore the Other Services section (New certificate · Revised certificate · Correction/Update · Withdraw) on the certificate page per the design.</t>
+        </is>
+      </c>
+      <c r="G21" s="24" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=3531-36666</t>
+        </is>
+      </c>
+      <c r="H21" s="24" t="inlineStr">
+        <is>
+          <t>https://tg-user-dev.mosje.in/certificate</t>
+        </is>
+      </c>
+      <c r="I21" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J21" s="23" t="inlineStr"/>
+      <c r="K21" s="23" t="inlineStr"/>
+      <c r="L21" s="23" t="inlineStr">
+        <is>
+          <t>env: dev</t>
+        </is>
+      </c>
+      <c r="M21" s="23" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>TG-CIT-CERT-DETAIL-002</t>
+        </is>
+      </c>
+      <c r="B22" s="21" t="inlineStr">
+        <is>
+          <t>Citizen — Certificate &amp; Identity Card</t>
+        </is>
+      </c>
+      <c r="C22" s="21" t="inlineStr">
+        <is>
+          <t>Typography</t>
+        </is>
+      </c>
+      <c r="D22" s="21" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E22" s="21" t="inlineStr">
+        <is>
+          <t>Figma: The page opens with the title 'Transgender Certificate &amp; Identity Card' and an explanatory paragraph about the certificate.  →  Live: The build starts straight at the approval card — no page title or intro copy.</t>
+        </is>
+      </c>
+      <c r="F22" s="21" t="inlineStr">
+        <is>
+          <t>Render the page title and intro paragraph per the design.</t>
+        </is>
+      </c>
+      <c r="G22" s="22" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=3531-36666</t>
+        </is>
+      </c>
+      <c r="H22" s="22" t="inlineStr">
+        <is>
+          <t>https://tg-user-dev.mosje.in/certificate</t>
+        </is>
+      </c>
+      <c r="I22" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J22" s="21" t="inlineStr"/>
+      <c r="K22" s="21" t="inlineStr"/>
+      <c r="L22" s="21" t="inlineStr">
+        <is>
+          <t>env: dev</t>
+        </is>
+      </c>
+      <c r="M22" s="21" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="23" t="inlineStr">
+        <is>
+          <t>TG-CIT-CERT-DETAIL-003</t>
+        </is>
+      </c>
+      <c r="B23" s="23" t="inlineStr">
+        <is>
+          <t>Citizen — Certificate &amp; Identity Card</t>
+        </is>
+      </c>
+      <c r="C23" s="23" t="inlineStr">
+        <is>
+          <t>Components &amp; States</t>
+        </is>
+      </c>
+      <c r="D23" s="23" t="inlineStr">
+        <is>
+          <t>Nit</t>
+        </is>
+      </c>
+      <c r="E23" s="23" t="inlineStr">
+        <is>
+          <t>Figma: The approval card offers 'Download Certificate' and 'Download ID Card'.  →  Live: The build offers 'Download Revised Certificate', 'Download ID Card', 'Gender Revision Request' and 'Collapse'.</t>
+        </is>
+      </c>
+      <c r="F23" s="23" t="inlineStr">
+        <is>
+          <t>Confirm the extra actions are intended and align the primary label with the design.</t>
+        </is>
+      </c>
+      <c r="G23" s="24" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=3531-36666</t>
+        </is>
+      </c>
+      <c r="H23" s="24" t="inlineStr">
+        <is>
+          <t>https://tg-user-dev.mosje.in/certificate</t>
+        </is>
+      </c>
+      <c r="I23" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J23" s="23" t="inlineStr"/>
+      <c r="K23" s="23" t="inlineStr"/>
+      <c r="L23" s="23" t="inlineStr">
+        <is>
+          <t>env: dev</t>
+        </is>
+      </c>
+      <c r="M23" s="23" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="21" t="inlineStr">
+        <is>
+          <t>TG-CIT-TRACK-001</t>
+        </is>
+      </c>
+      <c r="B24" s="21" t="inlineStr">
+        <is>
+          <t>Citizen — Track Status</t>
+        </is>
+      </c>
+      <c r="C24" s="21" t="inlineStr">
+        <is>
+          <t>Components &amp; States</t>
+        </is>
+      </c>
+      <c r="D24" s="21" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="E24" s="21" t="inlineStr">
+        <is>
+          <t>Figma: A Track page shows the application progress stepper (Submitted → In Scrutiny → Approval → Certificate Generation) with the current step highlighted, plus Withdraw Application, Correction Request and View Full Application actions.  →  Live: The build's track route renders the citizen dashboard instead — the progress stepper and its three actions do not exist anywhere in the build.</t>
+        </is>
+      </c>
+      <c r="F24" s="21" t="inlineStr">
+        <is>
+          <t>Build the track/status page per the design frame, including the progress stepper and the Withdraw / Correction Request / View Full Application actions.</t>
+        </is>
+      </c>
+      <c r="G24" s="22" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=3531-36747</t>
+        </is>
+      </c>
+      <c r="H24" s="22" t="inlineStr">
+        <is>
+          <t>https://tg-user-dev.mosje.in/track-status</t>
+        </is>
+      </c>
+      <c r="I24" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J24" s="21" t="inlineStr"/>
+      <c r="K24" s="21" t="inlineStr"/>
+      <c r="L24" s="21" t="inlineStr">
+        <is>
+          <t>env: dev</t>
+        </is>
+      </c>
+      <c r="M24" s="21" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t>TG-EOD-001</t>
+        </is>
+      </c>
+      <c r="B25" s="23" t="inlineStr">
+        <is>
+          <t>Examining Officer (Maker) — Dashboard</t>
+        </is>
+      </c>
+      <c r="C25" s="23" t="inlineStr">
+        <is>
+          <t>Components &amp; States</t>
+        </is>
+      </c>
+      <c r="D25" s="23" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E25" s="23" t="inlineStr">
+        <is>
+          <t>Figma: The design Maker queue has a Classification column (Clean / Exception badges) flagging exception applications.  →  Live: The build omits the Classification column, so triage exceptions aren't visible in the list.</t>
+        </is>
+      </c>
+      <c r="F25" s="23" t="inlineStr">
+        <is>
+          <t>Show the Classification column per the design (low priority — the build shows fewer columns than the design).</t>
+        </is>
+      </c>
+      <c r="G25" s="24" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-41744</t>
+        </is>
+      </c>
+      <c r="H25" s="24" t="inlineStr">
+        <is>
+          <t>https://tg-admin-dev.mosje.in/dashboard</t>
+        </is>
+      </c>
+      <c r="I25" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J25" s="23" t="inlineStr"/>
+      <c r="K25" s="23" t="inlineStr"/>
+      <c r="L25" s="23" t="inlineStr">
+        <is>
+          <t>env: dev</t>
+        </is>
+      </c>
+      <c r="M25" s="23" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>TG-EOD-002</t>
+        </is>
+      </c>
+      <c r="B26" s="21" t="inlineStr">
+        <is>
+          <t>Examining Officer (Maker) — Dashboard</t>
+        </is>
+      </c>
+      <c r="C26" s="21" t="inlineStr">
+        <is>
+          <t>Components &amp; States</t>
+        </is>
+      </c>
+      <c r="D26" s="21" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E26" s="21" t="inlineStr">
+        <is>
+          <t>Figma: The design queue header carries All Classifications / All Types / All Status filter dropdowns.  →  Live: The build has only a search box + a State/District toggle.</t>
+        </is>
+      </c>
+      <c r="F26" s="21" t="inlineStr">
+        <is>
+          <t>Surface the relevant queue filters per the design.</t>
+        </is>
+      </c>
+      <c r="G26" s="22" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-41744</t>
+        </is>
+      </c>
+      <c r="H26" s="22" t="inlineStr">
+        <is>
+          <t>https://tg-admin-dev.mosje.in/dashboard</t>
+        </is>
+      </c>
+      <c r="I26" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J26" s="21" t="inlineStr"/>
+      <c r="K26" s="21" t="inlineStr"/>
+      <c r="L26" s="21" t="inlineStr">
+        <is>
+          <t>env: dev</t>
+        </is>
+      </c>
+      <c r="M26" s="21" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="23" t="inlineStr">
+        <is>
+          <t>TG-DMD-001</t>
+        </is>
+      </c>
+      <c r="B27" s="23" t="inlineStr">
+        <is>
+          <t>District Magistrate — Dashboard</t>
+        </is>
+      </c>
+      <c r="C27" s="23" t="inlineStr">
+        <is>
+          <t>Components &amp; States</t>
+        </is>
+      </c>
+      <c r="D27" s="23" t="inlineStr">
+        <is>
+          <t>Nit</t>
+        </is>
+      </c>
+      <c r="E27" s="23" t="inlineStr">
+        <is>
+          <t>Figma: The design DM queue columns are Applicant ID, Name, District, Due in, Status.  →  Live: The build queue adds a 'Current Stage' column and a View action not in the design table.</t>
+        </is>
+      </c>
+      <c r="F27" s="23" t="inlineStr">
+        <is>
+          <t>Confirm if intended — the build has an extra column; do not remove without design sign-off.</t>
+        </is>
+      </c>
+      <c r="G27" s="24" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-42053</t>
+        </is>
+      </c>
+      <c r="H27" s="24" t="inlineStr">
+        <is>
+          <t>https://tg-admin-dev.mosje.in/dashboard</t>
+        </is>
+      </c>
+      <c r="I27" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J27" s="23" t="inlineStr"/>
+      <c r="K27" s="23" t="inlineStr"/>
+      <c r="L27" s="23" t="inlineStr">
+        <is>
+          <t>env: dev</t>
+        </is>
+      </c>
+      <c r="M27" s="23" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="21" t="inlineStr">
+        <is>
+          <t>TG-DM-MODAL-APPROVE-001</t>
+        </is>
+      </c>
+      <c r="B28" s="21" t="inlineStr">
+        <is>
+          <t>District Magistrate — Approve modal</t>
+        </is>
+      </c>
+      <c r="C28" s="21" t="inlineStr">
+        <is>
+          <t>Color &amp; Token</t>
+        </is>
+      </c>
+      <c r="D28" s="21" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E28" s="21" t="inlineStr">
+        <is>
+          <t>Figma: The applicant confirm box is green-tinted with a green border, reinforcing the approve action.  →  Live: The build renders a neutral grey box, losing the success affordance.</t>
+        </is>
+      </c>
+      <c r="F28" s="21" t="inlineStr">
+        <is>
+          <t>Apply the design's success tint + border to the applicant confirm box.</t>
+        </is>
+      </c>
+      <c r="G28" s="22" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-39988</t>
+        </is>
+      </c>
+      <c r="H28" s="22" t="inlineStr">
+        <is>
+          <t>https://tg-admin-dev.mosje.in/applications</t>
+        </is>
+      </c>
+      <c r="I28" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J28" s="21" t="inlineStr"/>
+      <c r="K28" s="21" t="inlineStr"/>
+      <c r="L28" s="21" t="inlineStr">
+        <is>
+          <t>env: dev</t>
+        </is>
+      </c>
+      <c r="M28" s="21" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="23" t="inlineStr">
+        <is>
+          <t>TG-DM-MODAL-APPROVE-002</t>
+        </is>
+      </c>
+      <c r="B29" s="23" t="inlineStr">
+        <is>
+          <t>District Magistrate — Approve modal</t>
+        </is>
+      </c>
+      <c r="C29" s="23" t="inlineStr">
+        <is>
+          <t>Content &amp; Iconography</t>
+        </is>
+      </c>
+      <c r="D29" s="23" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E29" s="23" t="inlineStr">
+        <is>
+          <t>Figma: The modal shows the applicant's photograph with a success check, so the approver can verify identity before committing.  →  Live: The build renders a generic placeholder avatar instead of the applicant's uploaded photo.</t>
+        </is>
+      </c>
+      <c r="F29" s="23" t="inlineStr">
+        <is>
+          <t>Render the applicant's photograph in the approve modal; confirm whether the placeholder is only a test-data artefact.</t>
+        </is>
+      </c>
+      <c r="G29" s="24" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-39988</t>
+        </is>
+      </c>
+      <c r="H29" s="24" t="inlineStr">
+        <is>
+          <t>https://tg-admin-dev.mosje.in/applications</t>
+        </is>
+      </c>
+      <c r="I29" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J29" s="23" t="inlineStr"/>
+      <c r="K29" s="23" t="inlineStr"/>
+      <c r="L29" s="23" t="inlineStr">
+        <is>
+          <t>env: dev</t>
+        </is>
+      </c>
+      <c r="M29" s="23" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="21" t="inlineStr">
+        <is>
+          <t>TG-DM-MODAL-APPROVE-003</t>
+        </is>
+      </c>
+      <c r="B30" s="21" t="inlineStr">
+        <is>
+          <t>District Magistrate — Approve modal</t>
+        </is>
+      </c>
+      <c r="C30" s="21" t="inlineStr">
+        <is>
+          <t>Components &amp; States</t>
+        </is>
+      </c>
+      <c r="D30" s="21" t="inlineStr">
+        <is>
+          <t>Nit</t>
+        </is>
+      </c>
+      <c r="E30" s="21" t="inlineStr">
+        <is>
+          <t>Figma: The approve modal has no remarks input.  →  Live: The build adds a 'Remarks (Optional)' textarea before the actions.</t>
+        </is>
+      </c>
+      <c r="F30" s="21" t="inlineStr">
+        <is>
+          <t>Confirm the remarks field is intended; if so, add it to the design frame.</t>
+        </is>
+      </c>
+      <c r="G30" s="22" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-39988</t>
+        </is>
+      </c>
+      <c r="H30" s="22" t="inlineStr">
+        <is>
+          <t>https://tg-admin-dev.mosje.in/applications</t>
+        </is>
+      </c>
+      <c r="I30" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J30" s="21" t="inlineStr"/>
+      <c r="K30" s="21" t="inlineStr"/>
+      <c r="L30" s="21" t="inlineStr">
+        <is>
+          <t>env: dev</t>
+        </is>
+      </c>
+      <c r="M30" s="21" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="23" t="inlineStr">
+        <is>
+          <t>TG-CAD-001</t>
+        </is>
+      </c>
+      <c r="B31" s="23" t="inlineStr">
+        <is>
+          <t>Central Admin — Dashboard</t>
+        </is>
+      </c>
+      <c r="C31" s="23" t="inlineStr">
+        <is>
+          <t>Layout &amp; Spacing</t>
+        </is>
+      </c>
+      <c r="D31" s="23" t="inlineStr">
+        <is>
+          <t>Nit</t>
+        </is>
+      </c>
+      <c r="E31" s="23" t="inlineStr">
+        <is>
+          <t>Figma: The design keeps the State / District / Date-range filters inside the Application Queue card.  →  Live: The build floats a global filter bar ABOVE the KPI cards; it is a richer analytics dashboard (6 KPIs + State/District charts) vs the design's 4-KPI exception queue.</t>
+        </is>
+      </c>
+      <c r="F31" s="23" t="inlineStr">
+        <is>
+          <t>Confirm the analytics layout is intended — the extra KPIs/charts are build-only (audit vs the visual language, don't remove).</t>
+        </is>
+      </c>
+      <c r="G31" s="24" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-38830</t>
+        </is>
+      </c>
+      <c r="H31" s="24" t="inlineStr">
+        <is>
+          <t>https://tg-admin-dev.mosje.in/dashboard</t>
+        </is>
+      </c>
+      <c r="I31" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J31" s="23" t="inlineStr"/>
+      <c r="K31" s="23" t="inlineStr"/>
+      <c r="L31" s="23" t="inlineStr">
+        <is>
+          <t>env: dev</t>
+        </is>
+      </c>
+      <c r="M31" s="23" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="21" t="inlineStr">
+        <is>
+          <t>TG-CAD-002</t>
+        </is>
+      </c>
+      <c r="B32" s="21" t="inlineStr">
+        <is>
+          <t>Central Admin — Dashboard</t>
+        </is>
+      </c>
+      <c r="C32" s="21" t="inlineStr">
+        <is>
+          <t>Color &amp; Token</t>
+        </is>
+      </c>
+      <c r="D32" s="21" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E32" s="21" t="inlineStr">
+        <is>
+          <t>Figma: Charts should use TG tokens — Primary/Source #003366 for bars, Success/Source #2e7d32 for the approval-rate series.  →  Live: Chart series may use raw greens/blues rather than the TG token palette.</t>
+        </is>
+      </c>
+      <c r="F32" s="21" t="inlineStr">
+        <is>
+          <t>Verify the chart palette against the TG tokens; the charts are a build-only section audited vs the visual language.</t>
+        </is>
+      </c>
+      <c r="G32" s="22" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-38830</t>
+        </is>
+      </c>
+      <c r="H32" s="22" t="inlineStr">
+        <is>
+          <t>https://tg-admin-dev.mosje.in/dashboard</t>
+        </is>
+      </c>
+      <c r="I32" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J32" s="21" t="inlineStr"/>
+      <c r="K32" s="21" t="inlineStr"/>
+      <c r="L32" s="21" t="inlineStr">
+        <is>
+          <t>env: dev</t>
+        </is>
+      </c>
+      <c r="M32" s="21" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="23" t="inlineStr">
+        <is>
+          <t>TG-AD-001</t>
+        </is>
+      </c>
+      <c r="B33" s="23" t="inlineStr">
+        <is>
+          <t>Admin — Application Detail</t>
+        </is>
+      </c>
+      <c r="C33" s="23" t="inlineStr">
+        <is>
+          <t>Layout &amp; Spacing</t>
+        </is>
+      </c>
+      <c r="D33" s="23" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E33" s="23" t="inlineStr">
+        <is>
+          <t>Figma: The design detail page is full-width (sidebar collapsed to a hamburger); the examining-officer / DM detail pages have no sidebar (match the design).  →  Live: The central-admin detail page keeps the admin sidebar expanded, narrowing the content column.</t>
+        </is>
+      </c>
+      <c r="F33" s="23" t="inlineStr">
+        <is>
+          <t>Confirm the central-admin sidebar on detail views is intended; otherwise collapse it to match the design.</t>
+        </is>
+      </c>
+      <c r="G33" s="24" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-38975</t>
+        </is>
+      </c>
+      <c r="H33" s="24" t="inlineStr">
+        <is>
+          <t>https://tg-admin-dev.mosje.in/applications</t>
+        </is>
+      </c>
+      <c r="I33" s="23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J33" s="23" t="inlineStr"/>
+      <c r="K33" s="23" t="inlineStr"/>
+      <c r="L33" s="23" t="inlineStr">
+        <is>
+          <t>env: dev</t>
+        </is>
+      </c>
+      <c r="M33" s="23" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="21" t="inlineStr">
+        <is>
+          <t>TG-AD-002</t>
+        </is>
+      </c>
+      <c r="B34" s="21" t="inlineStr">
+        <is>
+          <t>Admin — Application Detail</t>
+        </is>
+      </c>
+      <c r="C34" s="21" t="inlineStr">
+        <is>
+          <t>Components &amp; States</t>
+        </is>
+      </c>
+      <c r="D34" s="21" t="inlineStr">
+        <is>
+          <t>Nit</t>
+        </is>
+      </c>
+      <c r="E34" s="21" t="inlineStr">
+        <is>
+          <t>Figma: The design detail has 2 tabs: Applicant Details, Documents.  →  Live: The build has 4 tabs — it adds Revised Certificate and ID Card.</t>
+        </is>
+      </c>
+      <c r="F34" s="21" t="inlineStr">
+        <is>
+          <t>Build-extra — confirm if intended.</t>
+        </is>
+      </c>
+      <c r="G34" s="22" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-38975</t>
+        </is>
+      </c>
+      <c r="H34" s="22" t="inlineStr">
+        <is>
+          <t>https://tg-admin-dev.mosje.in/applications</t>
+        </is>
+      </c>
+      <c r="I34" s="21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="J34" s="21" t="inlineStr"/>
+      <c r="K34" s="21" t="inlineStr"/>
+      <c r="L34" s="21" t="inlineStr">
+        <is>
+          <t>env: dev</t>
+        </is>
+      </c>
+      <c r="M34" s="21" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:M34"/>
+  <dataValidations count="4">
+    <dataValidation sqref="D2:D400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Blocker,Major,Minor,Nit"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Layout &amp; Spacing,Color &amp; Token,Typography,Components &amp; States,Content &amp; Iconography,Responsive &amp; A11y"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Open,In Progress,Fixed,Won't Fix,Verified"</formula1>
+    </dataValidation>
+    <dataValidation sqref="M2:M400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Global,Screen"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H27" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H28" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H30" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H31" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H32" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H33" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H34" r:id="rId66"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>Screen</t>
+        </is>
+      </c>
+      <c r="B1" s="20" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="20" t="inlineStr">
+        <is>
+          <t>Figma URL</t>
+        </is>
+      </c>
+      <c r="D1" s="20" t="inlineStr">
+        <is>
+          <t>Has Design?</t>
+        </is>
+      </c>
+      <c r="E1" s="20" t="inlineStr">
+        <is>
+          <t>Built?</t>
+        </is>
+      </c>
+      <c r="F1" s="20" t="inlineStr">
+        <is>
+          <t>QC Status</t>
+        </is>
+      </c>
+      <c r="G1" s="20" t="inlineStr">
+        <is>
+          <t># Findings</t>
+        </is>
+      </c>
+      <c r="H1" s="20" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="21" t="inlineStr">
+        <is>
+          <t>Citizen — Sign In</t>
+        </is>
+      </c>
+      <c r="B2" s="21" t="inlineStr">
+        <is>
+          <t>Citizen</t>
+        </is>
+      </c>
+      <c r="C2" s="21" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=9379-115794</t>
+        </is>
+      </c>
+      <c r="D2" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E2" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F2" s="21" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="G2" s="21">
+        <f>COUNTIF('TG'!$B:$B,"Citizen — Sign In")</f>
+        <v/>
+      </c>
+      <c r="H2" s="21" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="23" t="inlineStr">
+        <is>
+          <t>Admin — Log In</t>
+        </is>
+      </c>
+      <c r="B3" s="23" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="C3" s="23" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=9387-138143</t>
+        </is>
+      </c>
+      <c r="D3" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E3" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F3" s="23" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="G3" s="23">
+        <f>COUNTIF('TG'!$B:$B,"Admin — Log In")</f>
+        <v/>
+      </c>
+      <c r="H3" s="23" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="21" t="inlineStr">
+        <is>
+          <t>Citizen — Apply · Pre-application</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>Citizen</t>
+        </is>
+      </c>
+      <c r="C4" s="21" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=3531-36958</t>
+        </is>
+      </c>
+      <c r="D4" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E4" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F4" s="21" t="inlineStr">
+        <is>
+          <t>Coverage — pending pins</t>
+        </is>
+      </c>
+      <c r="G4" s="21">
+        <f>COUNTIF('TG'!$B:$B,"Citizen — Apply · Pre-application")</f>
+        <v/>
+      </c>
+      <c r="H4" s="21" t="inlineStr">
+        <is>
+          <t>Portal-wide Global findings apply to this screen (masthead co-branding, KPI cards, tables, pagination — see the Global section). Design │ build shown for review; open the Figma frame ↗ for the intended design.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t>Citizen — Apply · Step 1 · Basic Identity Details</t>
+        </is>
+      </c>
+      <c r="B5" s="23" t="inlineStr">
+        <is>
+          <t>Citizen</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=3531-35553</t>
+        </is>
+      </c>
+      <c r="D5" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E5" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F5" s="23" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="G5" s="23">
+        <f>COUNTIF('TG'!$B:$B,"Citizen — Apply · Step 1 · Basic Identity Details")</f>
+        <v/>
+      </c>
+      <c r="H5" s="23" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>Citizen — Apply · Step 2 · Documents</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>Citizen</t>
+        </is>
+      </c>
+      <c r="C6" s="21" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=3531-35457</t>
+        </is>
+      </c>
+      <c r="D6" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E6" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F6" s="21" t="inlineStr">
+        <is>
+          <t>Coverage — pending pins</t>
+        </is>
+      </c>
+      <c r="G6" s="21">
+        <f>COUNTIF('TG'!$B:$B,"Citizen — Apply · Step 2 · Documents")</f>
+        <v/>
+      </c>
+      <c r="H6" s="21" t="inlineStr">
+        <is>
+          <t>Portal-wide Global findings apply to this screen (masthead co-branding, KPI cards, tables, pagination — see the Global section). Design │ build shown for review; open the Figma frame ↗ for the intended design.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t>Citizen — Apply · Step 3 · Review</t>
+        </is>
+      </c>
+      <c r="B7" s="23" t="inlineStr">
+        <is>
+          <t>Citizen</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=3531-35334</t>
+        </is>
+      </c>
+      <c r="D7" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E7" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F7" s="23" t="inlineStr">
+        <is>
+          <t>Coverage — pending pins</t>
+        </is>
+      </c>
+      <c r="G7" s="23">
+        <f>COUNTIF('TG'!$B:$B,"Citizen — Apply · Step 3 · Review")</f>
+        <v/>
+      </c>
+      <c r="H7" s="23" t="inlineStr">
+        <is>
+          <t>Portal-wide Global findings apply to this screen (masthead co-branding, KPI cards, tables, pagination — see the Global section). Design │ build shown for review; open the Figma frame ↗ for the intended design.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>Citizen — Apply · Confirmation</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>Citizen</t>
+        </is>
+      </c>
+      <c r="C8" s="21" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=3531-35271</t>
+        </is>
+      </c>
+      <c r="D8" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E8" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F8" s="21" t="inlineStr">
+        <is>
+          <t>Coverage — pending pins</t>
+        </is>
+      </c>
+      <c r="G8" s="21">
+        <f>COUNTIF('TG'!$B:$B,"Citizen — Apply · Confirmation")</f>
+        <v/>
+      </c>
+      <c r="H8" s="21" t="inlineStr">
+        <is>
+          <t>Portal-wide Global findings apply to this screen (masthead co-branding, KPI cards, tables, pagination — see the Global section). Design │ build shown for review; open the Figma frame ↗ for the intended design.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="23" t="inlineStr">
+        <is>
+          <t>Citizen — Dashboard · Certificate Active</t>
+        </is>
+      </c>
+      <c r="B9" s="23" t="inlineStr">
+        <is>
+          <t>Citizen</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=3531-36919</t>
+        </is>
+      </c>
+      <c r="D9" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E9" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F9" s="23" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="G9" s="23">
+        <f>COUNTIF('TG'!$B:$B,"Citizen — Dashboard · Certificate Active")</f>
+        <v/>
+      </c>
+      <c r="H9" s="23" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>Citizen — Certificate &amp; Identity Card</t>
+        </is>
+      </c>
+      <c r="B10" s="21" t="inlineStr">
+        <is>
+          <t>Citizen</t>
+        </is>
+      </c>
+      <c r="C10" s="21" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=3531-36666</t>
+        </is>
+      </c>
+      <c r="D10" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E10" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F10" s="21" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="G10" s="21">
+        <f>COUNTIF('TG'!$B:$B,"Citizen — Certificate &amp; Identity Card")</f>
+        <v/>
+      </c>
+      <c r="H10" s="21" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="23" t="inlineStr">
+        <is>
+          <t>Citizen — Certificate · ID Card</t>
+        </is>
+      </c>
+      <c r="B11" s="23" t="inlineStr">
+        <is>
+          <t>Citizen</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=3531-36841</t>
+        </is>
+      </c>
+      <c r="D11" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E11" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F11" s="23" t="inlineStr">
+        <is>
+          <t>Coverage — pending pins</t>
+        </is>
+      </c>
+      <c r="G11" s="23">
+        <f>COUNTIF('TG'!$B:$B,"Citizen — Certificate · ID Card")</f>
+        <v/>
+      </c>
+      <c r="H11" s="23" t="inlineStr">
+        <is>
+          <t>Portal-wide Global findings apply to this screen (masthead co-branding, KPI cards, tables, pagination — see the Global section). Design │ build shown for review; open the Figma frame ↗ for the intended design.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>Citizen — Track Status</t>
+        </is>
+      </c>
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>Citizen</t>
+        </is>
+      </c>
+      <c r="C12" s="21" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=3531-36747</t>
+        </is>
+      </c>
+      <c r="D12" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E12" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F12" s="21" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="G12" s="21">
+        <f>COUNTIF('TG'!$B:$B,"Citizen — Track Status")</f>
+        <v/>
+      </c>
+      <c r="H12" s="21" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="inlineStr">
+        <is>
+          <t>Citizen — Grievances</t>
+        </is>
+      </c>
+      <c r="B13" s="23" t="inlineStr">
+        <is>
+          <t>Citizen</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="inlineStr"/>
+      <c r="D13" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E13" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F13" s="23" t="inlineStr">
+        <is>
+          <t>Build-only</t>
+        </is>
+      </c>
+      <c r="G13" s="23">
+        <f>COUNTIF('TG'!$B:$B,"Citizen — Grievances")</f>
+        <v/>
+      </c>
+      <c r="H13" s="23" t="inlineStr">
+        <is>
+          <t>No design frame in the audited section — audited against the design-system visual language; the portal-wide Global findings apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="21" t="inlineStr">
+        <is>
+          <t>Examining Officer (Maker) — Dashboard</t>
+        </is>
+      </c>
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <t>Examining Officer (Maker)</t>
+        </is>
+      </c>
+      <c r="C14" s="21" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-41744</t>
+        </is>
+      </c>
+      <c r="D14" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E14" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F14" s="21" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="G14" s="21">
+        <f>COUNTIF('TG'!$B:$B,"Examining Officer (Maker) — Dashboard")</f>
+        <v/>
+      </c>
+      <c r="H14" s="21" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>Examining Officer (Maker) — Application Detail</t>
+        </is>
+      </c>
+      <c r="B15" s="23" t="inlineStr">
+        <is>
+          <t>Examining Officer (Maker)</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-38975</t>
+        </is>
+      </c>
+      <c r="D15" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E15" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F15" s="23" t="inlineStr">
+        <is>
+          <t>Coverage — pending pins</t>
+        </is>
+      </c>
+      <c r="G15" s="23">
+        <f>COUNTIF('TG'!$B:$B,"Examining Officer (Maker) — Application Detail")</f>
+        <v/>
+      </c>
+      <c r="H15" s="23" t="inlineStr">
+        <is>
+          <t>Portal-wide Global findings apply to this screen (masthead co-branding, KPI cards, tables, pagination — see the Global section). Design │ build shown for review; open the Figma frame ↗ for the intended design.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>Examining Officer (Maker) — Application Documents</t>
+        </is>
+      </c>
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>Examining Officer (Maker)</t>
+        </is>
+      </c>
+      <c r="C16" s="21" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-39123</t>
+        </is>
+      </c>
+      <c r="D16" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E16" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F16" s="21" t="inlineStr">
+        <is>
+          <t>Coverage — pending pins</t>
+        </is>
+      </c>
+      <c r="G16" s="21">
+        <f>COUNTIF('TG'!$B:$B,"Examining Officer (Maker) — Application Documents")</f>
+        <v/>
+      </c>
+      <c r="H16" s="21" t="inlineStr">
+        <is>
+          <t>Portal-wide Global findings apply to this screen (masthead co-branding, KPI cards, tables, pagination — see the Global section). Design │ build shown for review; open the Figma frame ↗ for the intended design.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="23" t="inlineStr">
+        <is>
+          <t>District Magistrate — Dashboard</t>
+        </is>
+      </c>
+      <c r="B17" s="23" t="inlineStr">
+        <is>
+          <t>District Magistrate</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-42053</t>
+        </is>
+      </c>
+      <c r="D17" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E17" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F17" s="23" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="G17" s="23">
+        <f>COUNTIF('TG'!$B:$B,"District Magistrate — Dashboard")</f>
+        <v/>
+      </c>
+      <c r="H17" s="23" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>District Magistrate — Application Detail · Actionable</t>
+        </is>
+      </c>
+      <c r="B18" s="21" t="inlineStr">
+        <is>
+          <t>District Magistrate</t>
+        </is>
+      </c>
+      <c r="C18" s="21" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-38975</t>
+        </is>
+      </c>
+      <c r="D18" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E18" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F18" s="21" t="inlineStr">
+        <is>
+          <t>Coverage — pending pins</t>
+        </is>
+      </c>
+      <c r="G18" s="21">
+        <f>COUNTIF('TG'!$B:$B,"District Magistrate — Application Detail · Actionable")</f>
+        <v/>
+      </c>
+      <c r="H18" s="21" t="inlineStr">
+        <is>
+          <t>Portal-wide Global findings apply to this screen (masthead co-branding, KPI cards, tables, pagination — see the Global section). Design │ build shown for review; open the Figma frame ↗ for the intended design.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="23" t="inlineStr">
+        <is>
+          <t>District Magistrate — Application Documents</t>
+        </is>
+      </c>
+      <c r="B19" s="23" t="inlineStr">
+        <is>
+          <t>District Magistrate</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-39123</t>
+        </is>
+      </c>
+      <c r="D19" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E19" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F19" s="23" t="inlineStr">
+        <is>
+          <t>Coverage — pending pins</t>
+        </is>
+      </c>
+      <c r="G19" s="23">
+        <f>COUNTIF('TG'!$B:$B,"District Magistrate — Application Documents")</f>
+        <v/>
+      </c>
+      <c r="H19" s="23" t="inlineStr">
+        <is>
+          <t>Portal-wide Global findings apply to this screen (masthead co-branding, KPI cards, tables, pagination — see the Global section). Design │ build shown for review; open the Figma frame ↗ for the intended design.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t>District Magistrate — Request-Correction modal</t>
+        </is>
+      </c>
+      <c r="B20" s="21" t="inlineStr">
+        <is>
+          <t>District Magistrate</t>
+        </is>
+      </c>
+      <c r="C20" s="21" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-39801</t>
+        </is>
+      </c>
+      <c r="D20" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E20" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F20" s="21" t="inlineStr">
+        <is>
+          <t>Coverage — pending pins</t>
+        </is>
+      </c>
+      <c r="G20" s="21">
+        <f>COUNTIF('TG'!$B:$B,"District Magistrate — Request-Correction modal")</f>
+        <v/>
+      </c>
+      <c r="H20" s="21" t="inlineStr">
+        <is>
+          <t>Portal-wide Global findings apply to this screen (masthead co-branding, KPI cards, tables, pagination — see the Global section). Design │ build shown for review; open the Figma frame ↗ for the intended design.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="23" t="inlineStr">
+        <is>
+          <t>District Magistrate — Approve modal</t>
+        </is>
+      </c>
+      <c r="B21" s="23" t="inlineStr">
+        <is>
+          <t>District Magistrate</t>
+        </is>
+      </c>
+      <c r="C21" s="23" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-39988</t>
+        </is>
+      </c>
+      <c r="D21" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E21" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F21" s="23" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="G21" s="23">
+        <f>COUNTIF('TG'!$B:$B,"District Magistrate — Approve modal")</f>
+        <v/>
+      </c>
+      <c r="H21" s="23" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>Central Admin — Dashboard</t>
+        </is>
+      </c>
+      <c r="B22" s="21" t="inlineStr">
+        <is>
+          <t>Central Admin</t>
+        </is>
+      </c>
+      <c r="C22" s="21" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-38830</t>
+        </is>
+      </c>
+      <c r="D22" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E22" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F22" s="21" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="G22" s="21">
+        <f>COUNTIF('TG'!$B:$B,"Central Admin — Dashboard")</f>
+        <v/>
+      </c>
+      <c r="H22" s="21" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="23" t="inlineStr">
+        <is>
+          <t>Admin — Application Detail</t>
+        </is>
+      </c>
+      <c r="B23" s="23" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="C23" s="23" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-38975</t>
+        </is>
+      </c>
+      <c r="D23" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E23" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F23" s="23" t="inlineStr">
+        <is>
+          <t>Reviewed</t>
+        </is>
+      </c>
+      <c r="G23" s="23">
+        <f>COUNTIF('TG'!$B:$B,"Admin — Application Detail")</f>
+        <v/>
+      </c>
+      <c r="H23" s="23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="21" t="inlineStr">
+        <is>
+          <t>Central Admin — Application Documents</t>
+        </is>
+      </c>
+      <c r="B24" s="21" t="inlineStr">
+        <is>
+          <t>Central Admin</t>
+        </is>
+      </c>
+      <c r="C24" s="21" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=2494-39123</t>
+        </is>
+      </c>
+      <c r="D24" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E24" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F24" s="21" t="inlineStr">
+        <is>
+          <t>Coverage — pending pins</t>
+        </is>
+      </c>
+      <c r="G24" s="21">
+        <f>COUNTIF('TG'!$B:$B,"Central Admin — Application Documents")</f>
+        <v/>
+      </c>
+      <c r="H24" s="21" t="inlineStr">
+        <is>
+          <t>Portal-wide Global findings apply to this screen (masthead co-branding, KPI cards, tables, pagination — see the Global section). Design │ build shown for review; open the Figma frame ↗ for the intended design.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t>District Magistrate — Reject modal (build-extra)</t>
+        </is>
+      </c>
+      <c r="B25" s="23" t="inlineStr">
+        <is>
+          <t>District Magistrate</t>
+        </is>
+      </c>
+      <c r="C25" s="23" t="inlineStr"/>
+      <c r="D25" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E25" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F25" s="23" t="inlineStr">
+        <is>
+          <t>Build-only</t>
+        </is>
+      </c>
+      <c r="G25" s="23">
+        <f>COUNTIF('TG'!$B:$B,"District Magistrate — Reject modal (build-extra)")</f>
+        <v/>
+      </c>
+      <c r="H25" s="23" t="inlineStr">
+        <is>
+          <t>No design frame in the audited section — audited against the design-system visual language; the portal-wide Global findings apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>Central Admin — User Management</t>
+        </is>
+      </c>
+      <c r="B26" s="21" t="inlineStr">
+        <is>
+          <t>Central Admin</t>
+        </is>
+      </c>
+      <c r="C26" s="21" t="inlineStr"/>
+      <c r="D26" s="21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E26" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F26" s="21" t="inlineStr">
+        <is>
+          <t>Build-only</t>
+        </is>
+      </c>
+      <c r="G26" s="21">
+        <f>COUNTIF('TG'!$B:$B,"Central Admin — User Management")</f>
+        <v/>
+      </c>
+      <c r="H26" s="21" t="inlineStr">
+        <is>
+          <t>No design frame in the audited section — audited against the design-system visual language; the portal-wide Global findings apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="23" t="inlineStr">
+        <is>
+          <t>Central Admin — Role Management</t>
+        </is>
+      </c>
+      <c r="B27" s="23" t="inlineStr">
+        <is>
+          <t>Central Admin</t>
+        </is>
+      </c>
+      <c r="C27" s="23" t="inlineStr"/>
+      <c r="D27" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E27" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F27" s="23" t="inlineStr">
+        <is>
+          <t>Build-only</t>
+        </is>
+      </c>
+      <c r="G27" s="23">
+        <f>COUNTIF('TG'!$B:$B,"Central Admin — Role Management")</f>
+        <v/>
+      </c>
+      <c r="H27" s="23" t="inlineStr">
+        <is>
+          <t>No design frame in the audited section — audited against the design-system visual language; the portal-wide Global findings apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="21" t="inlineStr">
+        <is>
+          <t>Central Admin — Tenants</t>
+        </is>
+      </c>
+      <c r="B28" s="21" t="inlineStr">
+        <is>
+          <t>Central Admin</t>
+        </is>
+      </c>
+      <c r="C28" s="21" t="inlineStr"/>
+      <c r="D28" s="21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E28" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F28" s="21" t="inlineStr">
+        <is>
+          <t>Build-only</t>
+        </is>
+      </c>
+      <c r="G28" s="21">
+        <f>COUNTIF('TG'!$B:$B,"Central Admin — Tenants")</f>
+        <v/>
+      </c>
+      <c r="H28" s="21" t="inlineStr">
+        <is>
+          <t>No design frame in the audited section — audited against the design-system visual language; the portal-wide Global findings apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="23" t="inlineStr">
+        <is>
+          <t>Central Admin — Password Policy</t>
+        </is>
+      </c>
+      <c r="B29" s="23" t="inlineStr">
+        <is>
+          <t>Central Admin</t>
+        </is>
+      </c>
+      <c r="C29" s="23" t="inlineStr"/>
+      <c r="D29" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E29" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F29" s="23" t="inlineStr">
+        <is>
+          <t>Build-only</t>
+        </is>
+      </c>
+      <c r="G29" s="23">
+        <f>COUNTIF('TG'!$B:$B,"Central Admin — Password Policy")</f>
+        <v/>
+      </c>
+      <c r="H29" s="23" t="inlineStr">
+        <is>
+          <t>No design frame in the audited section — audited against the design-system visual language; the portal-wide Global findings apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="21" t="inlineStr">
+        <is>
+          <t>All roles — Portal Picker (Change)</t>
+        </is>
+      </c>
+      <c r="B30" s="21" t="inlineStr">
+        <is>
+          <t>All roles</t>
+        </is>
+      </c>
+      <c r="C30" s="21" t="inlineStr">
+        <is>
+          <t>https://www.figma.com/design/gH2vQ62cfg4677YKWuOpLc/MoSJE-Portal--Handoff-?node-id=8103-39372</t>
+        </is>
+      </c>
+      <c r="D30" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E30" s="21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F30" s="21" t="inlineStr">
+        <is>
+          <t>Coverage — pending pins</t>
+        </is>
+      </c>
+      <c r="G30" s="21">
+        <f>COUNTIF('TG'!$B:$B,"All roles — Portal Picker (Change)")</f>
+        <v/>
+      </c>
+      <c r="H30" s="21" t="inlineStr">
+        <is>
+          <t>The '⇄ Change' button in the login footer opens this portal chooser. Verified faithful to the design (same 'Choose a portal to login' list + layout).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H30"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
chore(qc-tracker): bring the .xlsx trackers up to date with the live Google Sheet
The Drive Google Sheet and the .xlsx trackers had diverged in both directions.
The Sheet held work the spreadsheets had never seen — 43 NHAPOA findings marked
Fixed, and a hand-shortened fix text on NHA-GLOBAL-001. The spreadsheets held
tabs the Sheet has never had: the Coverage sheets, TG, and now SMILE Beggary.

So this is a merge, not a copy. sync_tracker_from_gsheet.py takes the Sheet
exported as .xlsx and brings cell values across for rows that exist in both,
keyed by finding ID; it never removes a row, a column or a tab, it skips Read Me
and Rollup (whose first column is not a finding id), it maps the Sheet's "NHAA"
tab to the file's "NHAPOA", and it reports every change before writing. Run it
without --apply for the dry run.

NHAPOA now reads 108 Open / 43 Fixed in both copies, matching the Sheet.
</commit_message>
<xml_diff>
--- a/docs/qc/MoSJE-Portal-QC-Tracker.xlsx
+++ b/docs/qc/MoSJE-Portal-QC-Tracker.xlsx
@@ -697,6 +697,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr"/>
       <c r="B4" s="4" t="inlineStr"/>
@@ -16472,7 +16473,7 @@
       </c>
       <c r="F2" s="21" t="inlineStr">
         <is>
-          <t>Restore the inline A−/A/A+ + contrast controls in the gov-bar on every page and trigger the UX4G widget from the bar's accessibility icon (not a floating FAB). Applies to every screen (citizen + admin).</t>
+          <t>Trigger the UX4G widget from the bar's accessibility icon (not a floating FAB). Applies to every screen (citizen + admin).</t>
         </is>
       </c>
       <c r="G2" s="22" t="inlineStr">
@@ -17313,7 +17314,7 @@
       </c>
       <c r="I16" s="21" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J16" s="21" t="inlineStr"/>
@@ -17372,7 +17373,7 @@
       </c>
       <c r="I17" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J17" s="23" t="inlineStr"/>
@@ -17431,7 +17432,7 @@
       </c>
       <c r="I18" s="21" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J18" s="21" t="inlineStr"/>
@@ -17490,7 +17491,7 @@
       </c>
       <c r="I19" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J19" s="23" t="inlineStr"/>
@@ -17549,7 +17550,7 @@
       </c>
       <c r="I20" s="21" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J20" s="21" t="inlineStr"/>
@@ -17608,7 +17609,7 @@
       </c>
       <c r="I21" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J21" s="23" t="inlineStr"/>
@@ -17667,7 +17668,7 @@
       </c>
       <c r="I22" s="21" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J22" s="21" t="inlineStr"/>
@@ -17726,7 +17727,7 @@
       </c>
       <c r="I23" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J23" s="23" t="inlineStr"/>
@@ -17785,7 +17786,7 @@
       </c>
       <c r="I24" s="21" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J24" s="21" t="inlineStr"/>
@@ -17844,7 +17845,7 @@
       </c>
       <c r="I25" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J25" s="23" t="inlineStr"/>
@@ -17903,7 +17904,7 @@
       </c>
       <c r="I26" s="21" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J26" s="21" t="inlineStr"/>
@@ -17962,7 +17963,7 @@
       </c>
       <c r="I27" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J27" s="23" t="inlineStr"/>
@@ -18021,7 +18022,7 @@
       </c>
       <c r="I28" s="21" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J28" s="21" t="inlineStr"/>
@@ -18080,7 +18081,7 @@
       </c>
       <c r="I29" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J29" s="23" t="inlineStr"/>
@@ -18139,7 +18140,7 @@
       </c>
       <c r="I30" s="21" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J30" s="21" t="inlineStr"/>
@@ -18198,7 +18199,7 @@
       </c>
       <c r="I31" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J31" s="23" t="inlineStr"/>
@@ -18257,7 +18258,7 @@
       </c>
       <c r="I32" s="21" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J32" s="21" t="inlineStr"/>
@@ -18316,7 +18317,7 @@
       </c>
       <c r="I33" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J33" s="23" t="inlineStr"/>
@@ -18375,7 +18376,7 @@
       </c>
       <c r="I34" s="21" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J34" s="21" t="inlineStr"/>
@@ -18434,7 +18435,7 @@
       </c>
       <c r="I35" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J35" s="23" t="inlineStr"/>
@@ -18493,7 +18494,7 @@
       </c>
       <c r="I36" s="21" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J36" s="21" t="inlineStr"/>
@@ -18552,7 +18553,7 @@
       </c>
       <c r="I37" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J37" s="23" t="inlineStr"/>
@@ -18611,7 +18612,7 @@
       </c>
       <c r="I38" s="21" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J38" s="21" t="inlineStr"/>
@@ -18670,7 +18671,7 @@
       </c>
       <c r="I39" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J39" s="23" t="inlineStr"/>
@@ -18729,7 +18730,7 @@
       </c>
       <c r="I40" s="21" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J40" s="21" t="inlineStr"/>
@@ -18784,7 +18785,7 @@
       </c>
       <c r="I41" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J41" s="23" t="inlineStr"/>
@@ -18839,7 +18840,7 @@
       </c>
       <c r="I42" s="21" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J42" s="21" t="inlineStr"/>
@@ -18894,7 +18895,7 @@
       </c>
       <c r="I43" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J43" s="23" t="inlineStr"/>
@@ -18949,7 +18950,7 @@
       </c>
       <c r="I44" s="21" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J44" s="21" t="inlineStr"/>
@@ -19008,7 +19009,7 @@
       </c>
       <c r="I45" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J45" s="23" t="inlineStr"/>
@@ -19067,7 +19068,7 @@
       </c>
       <c r="I46" s="21" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J46" s="21" t="inlineStr"/>
@@ -19126,7 +19127,7 @@
       </c>
       <c r="I47" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J47" s="23" t="inlineStr"/>
@@ -19185,7 +19186,7 @@
       </c>
       <c r="I48" s="21" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J48" s="21" t="inlineStr"/>
@@ -19244,7 +19245,7 @@
       </c>
       <c r="I49" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J49" s="23" t="inlineStr"/>
@@ -19303,7 +19304,7 @@
       </c>
       <c r="I50" s="21" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J50" s="21" t="inlineStr"/>
@@ -19362,7 +19363,7 @@
       </c>
       <c r="I51" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J51" s="23" t="inlineStr"/>
@@ -19417,7 +19418,7 @@
       </c>
       <c r="I52" s="21" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J52" s="21" t="inlineStr"/>
@@ -19472,7 +19473,7 @@
       </c>
       <c r="I53" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J53" s="23" t="inlineStr"/>
@@ -19527,7 +19528,7 @@
       </c>
       <c r="I54" s="21" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J54" s="21" t="inlineStr"/>
@@ -19582,7 +19583,7 @@
       </c>
       <c r="I55" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J55" s="23" t="inlineStr"/>
@@ -19637,7 +19638,7 @@
       </c>
       <c r="I56" s="21" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J56" s="21" t="inlineStr"/>
@@ -19692,7 +19693,7 @@
       </c>
       <c r="I57" s="23" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J57" s="23" t="inlineStr"/>
@@ -19747,7 +19748,7 @@
       </c>
       <c r="I58" s="21" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="J58" s="21" t="inlineStr"/>

</xml_diff>